<commit_message>
v38 study: orso Q11 accepts both b and c (stimulus says 'pesce' instead of 'pinnipede'), documented in limitations
- chiave_derivata.json: _accetta_anche mechanism; all scoring scripts updated
- pipeline rerun: main results unchanged (+1.4pt ns); orso Q11 no longer a problematic item
- CONCLUSIONI.md: added 'Limiti' section; INSIGHTS I-43 updated with the decision
- notebook regenerated and validated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/study/risultati_test.xlsx
+++ b/study/risultati_test.xlsx
@@ -692,10 +692,10 @@
         <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>64.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
@@ -2396,10 +2396,10 @@
         <v>14</v>
       </c>
       <c r="L27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
@@ -2408,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>50</v>
+        <v>57.1</v>
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         <v>14</v>
       </c>
       <c r="L49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
@@ -3970,11 +3970,11 @@
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="Q49" s="5" t="inlineStr">
-        <is>
-          <t>RAD</t>
+        <v>64.3</v>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>PSD</t>
         </is>
       </c>
     </row>
@@ -7749,10 +7749,10 @@
         <v>48</v>
       </c>
       <c r="C3" t="n">
-        <v>69.59999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>25.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -7765,10 +7765,10 @@
         <v>48</v>
       </c>
       <c r="C4" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="D4" t="n">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="6">
@@ -7798,7 +7798,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9">
@@ -7808,7 +7808,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.46</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="10">
@@ -7927,13 +7927,13 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>57.1</v>
+        <v>64.2</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>46.4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -8136,13 +8136,13 @@
         <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>66.09999999999999</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="D29" t="n">
         <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>65.7</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="31">
@@ -8212,10 +8212,10 @@
         <v>5</v>
       </c>
       <c r="C34" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E34" t="n">
         <v>7</v>
@@ -8356,10 +8356,10 @@
         <v>25</v>
       </c>
       <c r="C43" t="n">
-        <v>74.5</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D43" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="44">

</xml_diff>